<commit_message>
ATENÇÃO FASE 3 - REFATORADO PLANEJAMENTO
</commit_message>
<xml_diff>
--- a/projetos/OBRA_TMULT/03_PLANEJAMENTO_E_CRONOGRAMA/CRONOGRAMA_FISICO_FINANCEIRO_TMULT.xlsx
+++ b/projetos/OBRA_TMULT/03_PLANEJAMENTO_E_CRONOGRAMA/CRONOGRAMA_FISICO_FINANCEIRO_TMULT.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,12 +33,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00E8EEF5"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -79,8 +73,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F4F7"/>
-        <bgColor rgb="00F2F4F7"/>
+        <fgColor rgb="00F4F6F9"/>
+        <bgColor rgb="00F4F6F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -100,27 +94,27 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00DDDDDD"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00DDDDDD"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00DDDDDD"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00DDDDDD"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00DDDDDD"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00DDDDDD"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00DDDDDD"/>
       </top>
       <bottom style="double">
         <color rgb="001B365D"/>
@@ -133,41 +127,41 @@
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -726,7 +720,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OBRA TMULT — CRONOGRAMA FÍSICO-FINANCEIRO &amp; CURVA S</t>
+          <t>TMULT — TERMINAL MULTIUSO (PORTO DO AÇU) — EDIFÍCIO ADMINISTRATIVO — CRONOGRAMA FÍSICO-FINANCEIRO &amp; CURVA S</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(planejamento): implantacao da Fonte Unica da Verdade (SSOT) em JSON e motor compilar_planejamento
</commit_message>
<xml_diff>
--- a/projetos/OBRA_TMULT/03_PLANEJAMENTO_E_CRONOGRAMA/CRONOGRAMA_FISICO_FINANCEIRO_TMULT.xlsx
+++ b/projetos/OBRA_TMULT/03_PLANEJAMENTO_E_CRONOGRAMA/CRONOGRAMA_FISICO_FINANCEIRO_TMULT.xlsx
@@ -771,16 +771,16 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>163442.02</v>
+        <v>303629.55</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.09841385607577745</v>
+        <v>0.1828254131590706</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>163442.02</v>
+        <v>303629.55</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.09841385607577745</v>
+        <v>0.1828254131590706</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>0.1205</v>
@@ -793,10 +793,10 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>277895.85</v>
+        <v>137708.32</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>0.1673302996741954</v>
+        <v>0.08291874259090229</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>441337.87</v>
@@ -815,16 +815,16 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>347328.2</v>
+        <v>440941.88</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.2091378183276176</v>
+        <v>0.2655057170494022</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>788666.0699999999</v>
+        <v>882279.75</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.4748819740775905</v>
+        <v>0.5312498727993751</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>0.541</v>
@@ -837,16 +837,16 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>251786.96</v>
+        <v>271447.4</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.1516092718579808</v>
+        <v>0.1634474742526064</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>1040453.03</v>
+        <v>1153727.15</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>0.6264912459355713</v>
+        <v>0.6946973470519815</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>0.6984999999999999</v>
@@ -859,16 +859,16 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>333356.25</v>
+        <v>343651.97</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.200724844256458</v>
+        <v>0.2069242384286329</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1373809.28</v>
+        <v>1497379.12</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.8272160901920291</v>
+        <v>0.9016215854806144</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>0.884</v>
@@ -881,10 +881,10 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>286953</v>
+        <v>163383.16</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>0.1727839098079708</v>
+        <v>0.09837841451938564</v>
       </c>
       <c r="E11" s="8" t="n">
         <v>1660762.28</v>
@@ -2591,16 +2591,16 @@
         <v>5346.17</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>0</v>
+        <v>3742.32</v>
       </c>
       <c r="J26" s="9" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>5346.17</v>
+        <v>1603.85</v>
       </c>
       <c r="L26" s="9" t="n">
         <v>0</v>
@@ -2662,16 +2662,16 @@
         <v>15115.48</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>0</v>
+        <v>10580.84</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>15115.48</v>
+        <v>4534.64</v>
       </c>
       <c r="L27" s="6" t="n">
         <v>0</v>
@@ -2733,16 +2733,16 @@
         <v>15029.18</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>0</v>
+        <v>10520.43</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K28" s="8" t="n">
-        <v>15029.18</v>
+        <v>4508.75</v>
       </c>
       <c r="L28" s="9" t="n">
         <v>0</v>
@@ -2804,16 +2804,16 @@
         <v>30614.99</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>0</v>
+        <v>21430.49</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>30614.99</v>
+        <v>9184.5</v>
       </c>
       <c r="L29" s="6" t="n">
         <v>0</v>
@@ -2875,16 +2875,16 @@
         <v>11388.63</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I30" s="8" t="n">
-        <v>0</v>
+        <v>7972.04</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K30" s="8" t="n">
-        <v>11388.63</v>
+        <v>3416.59</v>
       </c>
       <c r="L30" s="9" t="n">
         <v>0</v>
@@ -2946,16 +2946,16 @@
         <v>32903.38</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>0</v>
+        <v>23032.37</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>32903.38</v>
+        <v>9871.01</v>
       </c>
       <c r="L31" s="6" t="n">
         <v>0</v>
@@ -3017,16 +3017,16 @@
         <v>20912.99</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>0</v>
+        <v>14639.09</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>20912.99</v>
+        <v>6273.9</v>
       </c>
       <c r="L32" s="9" t="n">
         <v>0</v>
@@ -3088,16 +3088,16 @@
         <v>32648.56</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>0</v>
+        <v>22853.99</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>32648.56</v>
+        <v>9794.57</v>
       </c>
       <c r="L33" s="6" t="n">
         <v>0</v>
@@ -3159,16 +3159,16 @@
         <v>149.24</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>0</v>
+        <v>104.47</v>
       </c>
       <c r="J34" s="9" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K34" s="8" t="n">
-        <v>149.24</v>
+        <v>44.77</v>
       </c>
       <c r="L34" s="9" t="n">
         <v>0</v>
@@ -3230,16 +3230,16 @@
         <v>24121.68</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>0</v>
+        <v>16885.18</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>24121.68</v>
+        <v>7236.5</v>
       </c>
       <c r="L35" s="6" t="n">
         <v>0</v>
@@ -3301,16 +3301,16 @@
         <v>12037.59</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>0</v>
+        <v>8426.309999999999</v>
       </c>
       <c r="J36" s="9" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>12037.59</v>
+        <v>3611.28</v>
       </c>
       <c r="L36" s="9" t="n">
         <v>0</v>
@@ -4313,16 +4313,16 @@
         <v>0</v>
       </c>
       <c r="N50" s="9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="O50" s="8" t="n">
-        <v>0</v>
+        <v>8084.54</v>
       </c>
       <c r="P50" s="9" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Q50" s="8" t="n">
-        <v>16169.08</v>
+        <v>8084.54</v>
       </c>
       <c r="R50" s="9" t="n">
         <v>0</v>
@@ -5384,16 +5384,16 @@
         <v>0</v>
       </c>
       <c r="P65" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q65" s="5" t="n">
-        <v>0</v>
+        <v>7916.96</v>
       </c>
       <c r="R65" s="6" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="S65" s="5" t="n">
-        <v>15833.91</v>
+        <v>7916.95</v>
       </c>
       <c r="T65" s="6">
         <f>H65+J65+L65+N65+P65+R65</f>
@@ -6792,16 +6792,16 @@
         <v>0</v>
       </c>
       <c r="L85" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M85" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N85" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O85" s="5" t="n">
         <v>3595.68</v>
-      </c>
-      <c r="N85" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O85" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="P85" s="6" t="n">
         <v>0</v>
@@ -6863,16 +6863,16 @@
         <v>0</v>
       </c>
       <c r="L86" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M86" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N86" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O86" s="8" t="n">
         <v>1765.4</v>
-      </c>
-      <c r="N86" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O86" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="P86" s="9" t="n">
         <v>0</v>
@@ -6934,16 +6934,16 @@
         <v>0</v>
       </c>
       <c r="L87" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M87" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N87" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O87" s="5" t="n">
         <v>140.8</v>
-      </c>
-      <c r="N87" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O87" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="P87" s="6" t="n">
         <v>0</v>
@@ -7005,16 +7005,16 @@
         <v>0</v>
       </c>
       <c r="L88" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M88" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N88" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O88" s="8" t="n">
         <v>217.44</v>
-      </c>
-      <c r="N88" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O88" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="P88" s="9" t="n">
         <v>0</v>
@@ -7147,16 +7147,16 @@
         <v>0</v>
       </c>
       <c r="L90" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M90" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N90" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O90" s="8" t="n">
         <v>6189.46</v>
-      </c>
-      <c r="N90" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O90" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="P90" s="9" t="n">
         <v>0</v>
@@ -7218,16 +7218,16 @@
         <v>0</v>
       </c>
       <c r="L91" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M91" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N91" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O91" s="5" t="n">
         <v>583.54</v>
-      </c>
-      <c r="N91" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O91" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="P91" s="6" t="n">
         <v>0</v>
@@ -7289,16 +7289,16 @@
         <v>0</v>
       </c>
       <c r="L92" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M92" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N92" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O92" s="8" t="n">
         <v>181.35</v>
-      </c>
-      <c r="N92" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O92" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="P92" s="9" t="n">
         <v>0</v>
@@ -7360,22 +7360,22 @@
         <v>0</v>
       </c>
       <c r="L93" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M93" s="5" t="n">
-        <v>488.32</v>
+        <v>0</v>
       </c>
       <c r="N93" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="O93" s="5" t="n">
-        <v>0</v>
+        <v>244.16</v>
       </c>
       <c r="P93" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q93" s="5" t="n">
-        <v>0</v>
+        <v>244.16</v>
       </c>
       <c r="R93" s="6" t="n">
         <v>0</v>
@@ -7431,22 +7431,22 @@
         <v>0</v>
       </c>
       <c r="L94" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M94" s="8" t="n">
-        <v>2960.71</v>
+        <v>0</v>
       </c>
       <c r="N94" s="9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="O94" s="8" t="n">
-        <v>0</v>
+        <v>1480.36</v>
       </c>
       <c r="P94" s="9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q94" s="8" t="n">
-        <v>0</v>
+        <v>1480.35</v>
       </c>
       <c r="R94" s="9" t="n">
         <v>0</v>
@@ -7502,10 +7502,10 @@
         <v>0</v>
       </c>
       <c r="L95" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M95" s="5" t="n">
-        <v>4169.02</v>
+        <v>0</v>
       </c>
       <c r="N95" s="6" t="n">
         <v>0</v>
@@ -7514,16 +7514,16 @@
         <v>0</v>
       </c>
       <c r="P95" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q95" s="5" t="n">
-        <v>0</v>
+        <v>2084.51</v>
       </c>
       <c r="R95" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="S95" s="5" t="n">
-        <v>0</v>
+        <v>2084.51</v>
       </c>
       <c r="T95" s="6">
         <f>H95+J95+L95+N95+P95+R95</f>
@@ -8295,16 +8295,16 @@
         <v>0</v>
       </c>
       <c r="P106" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q106" s="8" t="n">
-        <v>0</v>
+        <v>1989.04</v>
       </c>
       <c r="R106" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S106" s="8" t="n">
-        <v>1989.04</v>
+        <v>0</v>
       </c>
       <c r="T106" s="9">
         <f>H106+J106+L106+N106+P106+R106</f>
@@ -8792,16 +8792,16 @@
         <v>0</v>
       </c>
       <c r="P113" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q113" s="5" t="n">
-        <v>0</v>
+        <v>862.5</v>
       </c>
       <c r="R113" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S113" s="5" t="n">
-        <v>862.5</v>
+        <v>0</v>
       </c>
       <c r="T113" s="6">
         <f>H113+J113+L113+N113+P113+R113</f>
@@ -8863,16 +8863,16 @@
         <v>0</v>
       </c>
       <c r="P114" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q114" s="8" t="n">
-        <v>0</v>
+        <v>2662.9</v>
       </c>
       <c r="R114" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S114" s="8" t="n">
-        <v>2662.9</v>
+        <v>0</v>
       </c>
       <c r="T114" s="9">
         <f>H114+J114+L114+N114+P114+R114</f>
@@ -8934,16 +8934,16 @@
         <v>0</v>
       </c>
       <c r="P115" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q115" s="5" t="n">
-        <v>0</v>
+        <v>2817.5</v>
       </c>
       <c r="R115" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S115" s="5" t="n">
-        <v>2817.5</v>
+        <v>0</v>
       </c>
       <c r="T115" s="6">
         <f>H115+J115+L115+N115+P115+R115</f>
@@ -8999,22 +8999,22 @@
         <v>0</v>
       </c>
       <c r="N116" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O116" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P116" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q116" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R116" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S116" s="8" t="n">
         <v>1080.94</v>
-      </c>
-      <c r="P116" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q116" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R116" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="S116" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="T116" s="9">
         <f>H116+J116+L116+N116+P116+R116</f>
@@ -9070,22 +9070,22 @@
         <v>0</v>
       </c>
       <c r="N117" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O117" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P117" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q117" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R117" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S117" s="5" t="n">
         <v>1611.58</v>
-      </c>
-      <c r="P117" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q117" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R117" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S117" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="T117" s="6">
         <f>H117+J117+L117+N117+P117+R117</f>
@@ -9141,10 +9141,10 @@
         <v>0</v>
       </c>
       <c r="N118" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O118" s="8" t="n">
-        <v>0</v>
+        <v>534.11</v>
       </c>
       <c r="P118" s="9" t="n">
         <v>0</v>
@@ -9153,10 +9153,10 @@
         <v>0</v>
       </c>
       <c r="R118" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S118" s="8" t="n">
-        <v>534.11</v>
+        <v>0</v>
       </c>
       <c r="T118" s="9">
         <f>H118+J118+L118+N118+P118+R118</f>
@@ -9218,16 +9218,16 @@
         <v>0</v>
       </c>
       <c r="P119" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q119" s="5" t="n">
-        <v>0</v>
+        <v>673.12</v>
       </c>
       <c r="R119" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S119" s="5" t="n">
-        <v>673.12</v>
+        <v>0</v>
       </c>
       <c r="T119" s="6">
         <f>H119+J119+L119+N119+P119+R119</f>
@@ -9289,16 +9289,16 @@
         <v>0</v>
       </c>
       <c r="P120" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q120" s="8" t="n">
-        <v>0</v>
+        <v>1190.34</v>
       </c>
       <c r="R120" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S120" s="8" t="n">
-        <v>1190.34</v>
+        <v>0</v>
       </c>
       <c r="T120" s="9">
         <f>H120+J120+L120+N120+P120+R120</f>
@@ -9431,16 +9431,16 @@
         <v>0</v>
       </c>
       <c r="P122" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q122" s="8" t="n">
-        <v>0</v>
+        <v>691.84</v>
       </c>
       <c r="R122" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S122" s="8" t="n">
-        <v>691.84</v>
+        <v>0</v>
       </c>
       <c r="T122" s="9">
         <f>H122+J122+L122+N122+P122+R122</f>
@@ -9502,16 +9502,16 @@
         <v>0</v>
       </c>
       <c r="P123" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q123" s="5" t="n">
-        <v>0</v>
+        <v>6788.44</v>
       </c>
       <c r="R123" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S123" s="5" t="n">
-        <v>6788.44</v>
+        <v>0</v>
       </c>
       <c r="T123" s="6">
         <f>H123+J123+L123+N123+P123+R123</f>
@@ -9573,16 +9573,16 @@
         <v>0</v>
       </c>
       <c r="P124" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q124" s="8" t="n">
-        <v>0</v>
+        <v>2340</v>
       </c>
       <c r="R124" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S124" s="8" t="n">
-        <v>2340</v>
+        <v>0</v>
       </c>
       <c r="T124" s="9">
         <f>H124+J124+L124+N124+P124+R124</f>
@@ -9644,16 +9644,16 @@
         <v>0</v>
       </c>
       <c r="P125" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q125" s="5" t="n">
-        <v>0</v>
+        <v>1103.9</v>
       </c>
       <c r="R125" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S125" s="5" t="n">
-        <v>1103.9</v>
+        <v>0</v>
       </c>
       <c r="T125" s="6">
         <f>H125+J125+L125+N125+P125+R125</f>
@@ -10206,16 +10206,16 @@
         <v>0</v>
       </c>
       <c r="N133" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O133" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P133" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q133" s="5" t="n">
         <v>202.1</v>
-      </c>
-      <c r="P133" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q133" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="R133" s="6" t="n">
         <v>0</v>
@@ -10277,16 +10277,16 @@
         <v>0</v>
       </c>
       <c r="N134" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O134" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P134" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q134" s="8" t="n">
         <v>211.52</v>
-      </c>
-      <c r="P134" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q134" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="R134" s="9" t="n">
         <v>0</v>
@@ -10348,16 +10348,16 @@
         <v>0</v>
       </c>
       <c r="N135" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O135" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P135" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q135" s="5" t="n">
         <v>207.6</v>
-      </c>
-      <c r="P135" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q135" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="R135" s="6" t="n">
         <v>0</v>
@@ -10419,16 +10419,16 @@
         <v>0</v>
       </c>
       <c r="N136" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O136" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P136" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q136" s="8" t="n">
         <v>177.12</v>
-      </c>
-      <c r="P136" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q136" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="R136" s="9" t="n">
         <v>0</v>
@@ -10490,16 +10490,16 @@
         <v>0</v>
       </c>
       <c r="N137" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P137" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q137" s="5" t="n">
         <v>194.58</v>
-      </c>
-      <c r="P137" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q137" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="R137" s="6" t="n">
         <v>0</v>
@@ -10561,16 +10561,16 @@
         <v>0</v>
       </c>
       <c r="N138" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O138" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P138" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q138" s="8" t="n">
         <v>110.32</v>
-      </c>
-      <c r="P138" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q138" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="R138" s="9" t="n">
         <v>0</v>
@@ -10916,22 +10916,22 @@
         <v>0</v>
       </c>
       <c r="N143" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P143" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R143" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S143" s="5" t="n">
         <v>1278.72</v>
-      </c>
-      <c r="P143" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q143" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R143" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S143" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="T143" s="6">
         <f>H143+J143+L143+N143+P143+R143</f>
@@ -10987,22 +10987,22 @@
         <v>0</v>
       </c>
       <c r="N144" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O144" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P144" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q144" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R144" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S144" s="8" t="n">
         <v>722.3200000000001</v>
-      </c>
-      <c r="P144" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q144" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R144" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="S144" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="T144" s="9">
         <f>H144+J144+L144+N144+P144+R144</f>
@@ -11058,22 +11058,22 @@
         <v>0</v>
       </c>
       <c r="N145" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P145" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R145" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S145" s="5" t="n">
         <v>522.66</v>
-      </c>
-      <c r="P145" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q145" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R145" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S145" s="5" t="n">
-        <v>0</v>
       </c>
       <c r="T145" s="6">
         <f>H145+J145+L145+N145+P145+R145</f>
@@ -11129,16 +11129,16 @@
         <v>0</v>
       </c>
       <c r="N146" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O146" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P146" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q146" s="8" t="n">
         <v>216.18</v>
-      </c>
-      <c r="P146" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q146" s="8" t="n">
-        <v>0</v>
       </c>
       <c r="R146" s="9" t="n">
         <v>0</v>
@@ -11206,16 +11206,16 @@
         <v>0</v>
       </c>
       <c r="P147" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q147" s="5" t="n">
-        <v>0</v>
+        <v>6095</v>
       </c>
       <c r="R147" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S147" s="5" t="n">
-        <v>6095</v>
+        <v>0</v>
       </c>
       <c r="T147" s="6">
         <f>H147+J147+L147+N147+P147+R147</f>
@@ -11277,16 +11277,16 @@
         <v>0</v>
       </c>
       <c r="P148" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q148" s="8" t="n">
-        <v>0</v>
+        <v>863.52</v>
       </c>
       <c r="R148" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S148" s="8" t="n">
-        <v>863.52</v>
+        <v>0</v>
       </c>
       <c r="T148" s="9">
         <f>H148+J148+L148+N148+P148+R148</f>
@@ -11342,10 +11342,10 @@
         <v>0</v>
       </c>
       <c r="N149" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O149" s="5" t="n">
-        <v>0</v>
+        <v>966.5</v>
       </c>
       <c r="P149" s="6" t="n">
         <v>0</v>
@@ -11354,10 +11354,10 @@
         <v>0</v>
       </c>
       <c r="R149" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S149" s="5" t="n">
-        <v>966.5</v>
+        <v>0</v>
       </c>
       <c r="T149" s="6">
         <f>H149+J149+L149+N149+P149+R149</f>
@@ -11413,10 +11413,10 @@
         <v>0</v>
       </c>
       <c r="N150" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O150" s="8" t="n">
-        <v>0</v>
+        <v>2212.74</v>
       </c>
       <c r="P150" s="9" t="n">
         <v>0</v>
@@ -11425,10 +11425,10 @@
         <v>0</v>
       </c>
       <c r="R150" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S150" s="8" t="n">
-        <v>2212.74</v>
+        <v>0</v>
       </c>
       <c r="T150" s="9">
         <f>H150+J150+L150+N150+P150+R150</f>
@@ -11632,16 +11632,16 @@
         <v>0</v>
       </c>
       <c r="P153" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q153" s="5" t="n">
-        <v>0</v>
+        <v>258.16</v>
       </c>
       <c r="R153" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S153" s="5" t="n">
-        <v>258.16</v>
+        <v>0</v>
       </c>
       <c r="T153" s="6">
         <f>H153+J153+L153+N153+P153+R153</f>
@@ -11703,16 +11703,16 @@
         <v>0</v>
       </c>
       <c r="P154" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q154" s="8" t="n">
-        <v>0</v>
+        <v>615.5599999999999</v>
       </c>
       <c r="R154" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S154" s="8" t="n">
-        <v>615.5599999999999</v>
+        <v>0</v>
       </c>
       <c r="T154" s="9">
         <f>H154+J154+L154+N154+P154+R154</f>
@@ -11774,16 +11774,16 @@
         <v>0</v>
       </c>
       <c r="P155" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q155" s="5" t="n">
-        <v>0</v>
+        <v>427.32</v>
       </c>
       <c r="R155" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S155" s="5" t="n">
-        <v>427.32</v>
+        <v>0</v>
       </c>
       <c r="T155" s="6">
         <f>H155+J155+L155+N155+P155+R155</f>
@@ -11845,16 +11845,16 @@
         <v>0</v>
       </c>
       <c r="P156" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q156" s="8" t="n">
-        <v>0</v>
+        <v>129.72</v>
       </c>
       <c r="R156" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S156" s="8" t="n">
-        <v>129.72</v>
+        <v>0</v>
       </c>
       <c r="T156" s="9">
         <f>H156+J156+L156+N156+P156+R156</f>
@@ -11904,10 +11904,10 @@
         <v>0</v>
       </c>
       <c r="L157" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M157" s="5" t="n">
-        <v>0</v>
+        <v>47274.56</v>
       </c>
       <c r="N157" s="6" t="n">
         <v>0</v>
@@ -11922,10 +11922,10 @@
         <v>0</v>
       </c>
       <c r="R157" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S157" s="5" t="n">
-        <v>47274.56</v>
+        <v>0</v>
       </c>
       <c r="T157" s="6">
         <f>H157+J157+L157+N157+P157+R157</f>
@@ -11975,10 +11975,10 @@
         <v>0</v>
       </c>
       <c r="L158" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M158" s="8" t="n">
-        <v>0</v>
+        <v>25045.98</v>
       </c>
       <c r="N158" s="9" t="n">
         <v>0</v>
@@ -11993,10 +11993,10 @@
         <v>0</v>
       </c>
       <c r="R158" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S158" s="8" t="n">
-        <v>25045.98</v>
+        <v>0</v>
       </c>
       <c r="T158" s="9">
         <f>H158+J158+L158+N158+P158+R158</f>
@@ -12046,10 +12046,10 @@
         <v>0</v>
       </c>
       <c r="L159" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M159" s="5" t="n">
-        <v>0</v>
+        <v>17410.86</v>
       </c>
       <c r="N159" s="6" t="n">
         <v>0</v>
@@ -12064,10 +12064,10 @@
         <v>0</v>
       </c>
       <c r="R159" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S159" s="5" t="n">
-        <v>17410.86</v>
+        <v>0</v>
       </c>
       <c r="T159" s="6">
         <f>H159+J159+L159+N159+P159+R159</f>
@@ -12117,10 +12117,10 @@
         <v>0</v>
       </c>
       <c r="L160" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M160" s="8" t="n">
-        <v>0</v>
+        <v>18885.6</v>
       </c>
       <c r="N160" s="9" t="n">
         <v>0</v>
@@ -12129,10 +12129,10 @@
         <v>0</v>
       </c>
       <c r="P160" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q160" s="8" t="n">
-        <v>18885.6</v>
+        <v>0</v>
       </c>
       <c r="R160" s="9" t="n">
         <v>0</v>
@@ -12188,10 +12188,10 @@
         <v>0</v>
       </c>
       <c r="L161" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M161" s="5" t="n">
-        <v>0</v>
+        <v>3770.4</v>
       </c>
       <c r="N161" s="6" t="n">
         <v>0</v>
@@ -12200,10 +12200,10 @@
         <v>0</v>
       </c>
       <c r="P161" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q161" s="5" t="n">
-        <v>3770.4</v>
+        <v>0</v>
       </c>
       <c r="R161" s="6" t="n">
         <v>0</v>
@@ -12259,10 +12259,10 @@
         <v>0</v>
       </c>
       <c r="L162" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M162" s="8" t="n">
-        <v>0</v>
+        <v>1518</v>
       </c>
       <c r="N162" s="9" t="n">
         <v>0</v>
@@ -12271,10 +12271,10 @@
         <v>0</v>
       </c>
       <c r="P162" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q162" s="8" t="n">
-        <v>1518</v>
+        <v>0</v>
       </c>
       <c r="R162" s="9" t="n">
         <v>0</v>

</xml_diff>